<commit_message>
feat: AI Templates & add bug screenshot on github repo & adjust test case
</commit_message>
<xml_diff>
--- a/Test_Cases.xlsx
+++ b/Test_Cases.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DAIHOC\KiemThuPM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DaiHoc\KiemThuPM\HW01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F7874FFD-271A-47C2-81BF-D89FF4377263}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D383E47A-FB71-4679-9F00-8B5516940DD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8C368C04-6EE2-4CEA-A1F8-4B04B0094A9B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8C368C04-6EE2-4CEA-A1F8-4B04B0094A9B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -288,9 +288,6 @@
     <t>Nút 1 bị đẩy nảy lên, ngắt điện động cơ ngay cả khi nút 0 chưa lún hoàn toàn xuống rãnh khóa.</t>
   </si>
   <si>
-    <t>Động cơ phát ra tiếng "è è" nhưng không cháy động cơ. Khi rút đũa thì quạt quay bình thường và ổn định.</t>
-  </si>
-  <si>
     <t>Quạt phát ra tiếng "cạch cạch" ở hộp số đằng sau và khi thả tay ra, quạt vẫn xoay bình thường và ổn định.</t>
   </si>
   <si>
@@ -330,13 +327,16 @@
     <t>Nút 1 nảy lên ngay khi nút 0 chưa lún xuống hoàn toàn, quạt ngừng quay.</t>
   </si>
   <si>
-    <t>Động cơ quạt phát ra tiếng "è è", không thấy cháy động cơ. Rút đũa thì quay lấy lại tốc độ và quay bình thường, ổn định.</t>
-  </si>
-  <si>
     <t>Quạt phát ra tiếng "cạch cạch" khi bị chặn lại và quạt quay bình thường, ổn định khi thả tay ra.</t>
   </si>
   <si>
     <t>Sau khi buông tay, quạt tự lấy lại cân bằng (thẳng đứng) và vẫn quay ổn định</t>
+  </si>
+  <si>
+    <t>Động cơ không phát ra tiếng, không bị cháy hay nóng và không quay. Khi rút đũa thì quạt quay bình thường và ổn định.</t>
+  </si>
+  <si>
+    <t>Động cơ quạt không phát ra tiếng, không thấy cháy động cơ và không có quay. Rút đũa thì quạt lấy lại tốc độ và quay bình thường, ổn định.</t>
   </si>
 </sst>
 </file>
@@ -472,7 +472,7 @@
   <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -487,7 +487,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -508,10 +508,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -849,19 +849,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9BAE0FEA-C4CD-4B67-8CBA-D558C2923CD9}">
   <dimension ref="A1:G16"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.77734375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="42.77734375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="15.5546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="48.44140625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="24.88671875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="22.33203125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="9.77734375" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.88671875" style="1"/>
+    <col min="1" max="1" width="13.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="42.7109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="15.5703125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="48.42578125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="24.85546875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="22.28515625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="9.7109375" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -884,7 +884,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="62.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="63" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>7</v>
       </c>
@@ -907,7 +907,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>14</v>
       </c>
@@ -924,13 +924,13 @@
         <v>65</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G3" s="8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="62.4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" ht="63" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
         <v>15</v>
       </c>
@@ -947,13 +947,13 @@
         <v>66</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G4" s="8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="78" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="78.75" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
         <v>16</v>
       </c>
@@ -970,13 +970,13 @@
         <v>67</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G5" s="8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
         <v>17</v>
       </c>
@@ -993,13 +993,13 @@
         <v>68</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G6" s="8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="62.4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" ht="63" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
         <v>18</v>
       </c>
@@ -1016,13 +1016,13 @@
         <v>69</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G7" s="8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="62.4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" ht="63" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
         <v>19</v>
       </c>
@@ -1039,13 +1039,13 @@
         <v>70</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G8" s="8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="78" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" ht="78.75" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
         <v>20</v>
       </c>
@@ -1062,13 +1062,13 @@
         <v>71</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G9" s="8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
         <v>21</v>
       </c>
@@ -1085,13 +1085,13 @@
         <v>72</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G10" s="8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
         <v>22</v>
       </c>
@@ -1108,13 +1108,13 @@
         <v>73</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G11" s="8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="62.4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" ht="63" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
         <v>23</v>
       </c>
@@ -1131,13 +1131,13 @@
         <v>74</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G12" s="8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="62.4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" ht="63" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>24</v>
       </c>
@@ -1154,13 +1154,13 @@
         <v>75</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G13" s="8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="93.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" ht="110.25" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
         <v>25</v>
       </c>
@@ -1174,16 +1174,16 @@
         <v>62</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>76</v>
+        <v>91</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="G14" s="8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="78" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" ht="78.75" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
         <v>26</v>
       </c>
@@ -1197,16 +1197,16 @@
         <v>63</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="G15" s="8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="62.4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" ht="63" x14ac:dyDescent="0.25">
       <c r="A16" s="15" t="s">
         <v>27</v>
       </c>
@@ -1220,10 +1220,10 @@
         <v>64</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="G16" s="11" t="s">
         <v>12</v>

</xml_diff>